<commit_message>
docs(plan): link milestone sheet to GitHub issues, milestones and board
Every task row now links its GitHub issue (#186–#349), every milestone
links its GitHub milestone, and both docs point at the
"TaqatSpace Roadmap" project board.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DOCS/new plan/TaqatSpace-Milestone-Sheet.xlsx
+++ b/DOCS/new plan/TaqatSpace-Milestone-Sheet.xlsx
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Questions" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$1:$L$165</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$1:$M$165</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Gap Matrix'!$A$1:$F$137</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,7 +29,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +56,12 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="4">
@@ -102,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" readingOrder="2"/>
@@ -142,6 +148,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -535,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -559,47 +568,47 @@
       <c r="A3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>الحالة الحية لكل مهمة على GitHub (Issue لكل مهمة + لوحة Project «TaqatSpace Roadmap»)؛ هذا الملف لقطة للتخطيط والجهد. عمود Issue يفتح المهمة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>طريقة الاستخدام:</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>1) في ورقة Tasks عدّل فقط الأعمدة المظللة بالأصفر: «الحالة» (قائمة منسدلة) و«الفرع» و«PR» و«ملاحظات».</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>2) ورقة Summary تحسب الجهد والمدة ونسبة الإنجاز تلقائيًا بالمعادلات — لا تكتب فيها يدويًا.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>3) الجهد بأيام عمل لمطوّر واحد + Claude؛ المدة = الجهد ÷ 5 أيام.</t>
+          <t>1) في ورقة Tasks عدّل فقط الأعمدة المظللة بالأصفر: «الحالة» (قائمة منسدلة) و«الفرع» و«PR» و«ملاحظات».</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>4) «قابلة للتأجيل = نعم» تعني أن المهمة خارج المسار الأدنى للانتقال.</t>
+          <t>2) ورقة Summary تحسب الجهد والمدة ونسبة الإنجاز تلقائيًا بالمعادلات — لا تكتب فيها يدويًا.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>3) الجهد بأيام عمل لمطوّر واحد + Claude؛ المدة = الجهد ÷ 5 أيام.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>مثال لصف مكتمل: الحالة = «✅ مكتمل»، الفرع = feat/m2-mikrotik-sync، PR = #190.</t>
+          <t>4) «قابلة للتأجيل = نعم» تعني أن المهمة خارج المسار الأدنى للانتقال.</t>
         </is>
       </c>
     </row>
@@ -609,19 +618,29 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>مفتاح الحالة: ⬜ لم يبدأ · 🟨 قيد التنفيذ · ✅ مكتمل · ⛔ متوقف</t>
+          <t>مثال لصف مكتمل: الحالة = «✅ مكتمل»، الفرع = feat/m2-mikrotik-sync، PR = #190.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>مفتاح الوضع الحالي: جديد / توسعة (كود قائم يُبنى عليه) / موجود (ربط ومراجعة فقط)</t>
-        </is>
-      </c>
+      <c r="A13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>مفتاح الحالة: ⬜ لم يبدأ · 🟨 قيد التنفيذ · ✅ مكتمل · ⛔ متوقف</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>مفتاح الوضع الحالي: جديد / توسعة (كود قائم يُبنى عليه) / موجود (ربط ومراجعة فقط)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>مصدر التقديرات: تقدير أولي ±20% من فريق التطوير (2026-10-29)، يُعاد ضبطه بعد M2.</t>
         </is>
@@ -1412,7 +1431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L165"/>
+  <dimension ref="A1:M165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1424,9 +1443,10 @@
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1490,6 +1510,11 @@
           <t>ملاحظات</t>
         </is>
       </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -1537,11 +1562,16 @@
       </c>
       <c r="J2" s="14" t="inlineStr">
         <is>
-          <t>chore/m0-stabilize</t>
+          <t>chore/m0-1</t>
         </is>
       </c>
       <c r="K2" s="14" t="inlineStr"/>
       <c r="L2" s="14" t="inlineStr"/>
+      <c r="M2" s="15" t="inlineStr">
+        <is>
+          <t>#186</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -1589,11 +1619,16 @@
       </c>
       <c r="J3" s="14" t="inlineStr">
         <is>
-          <t>chore/m0-stabilize</t>
+          <t>chore/m0-2</t>
         </is>
       </c>
       <c r="K3" s="14" t="inlineStr"/>
       <c r="L3" s="14" t="inlineStr"/>
+      <c r="M3" s="15" t="inlineStr">
+        <is>
+          <t>#187</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -1641,11 +1676,16 @@
       </c>
       <c r="J4" s="14" t="inlineStr">
         <is>
-          <t>chore/m0-stabilize</t>
+          <t>chore/m0-3</t>
         </is>
       </c>
       <c r="K4" s="14" t="inlineStr"/>
       <c r="L4" s="14" t="inlineStr"/>
+      <c r="M4" s="15" t="inlineStr">
+        <is>
+          <t>#188</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -1693,11 +1733,16 @@
       </c>
       <c r="J5" s="14" t="inlineStr">
         <is>
-          <t>chore/m0-stabilize</t>
+          <t>chore/m0-4</t>
         </is>
       </c>
       <c r="K5" s="14" t="inlineStr"/>
       <c r="L5" s="14" t="inlineStr"/>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>#189</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1745,11 +1790,16 @@
       </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>chore/m0-stabilize</t>
+          <t>chore/m0-5</t>
         </is>
       </c>
       <c r="K6" s="14" t="inlineStr"/>
       <c r="L6" s="14" t="inlineStr"/>
+      <c r="M6" s="15" t="inlineStr">
+        <is>
+          <t>#190</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -1797,11 +1847,16 @@
       </c>
       <c r="J7" s="14" t="inlineStr">
         <is>
-          <t>chore/m0-stabilize</t>
+          <t>chore/m0-6</t>
         </is>
       </c>
       <c r="K7" s="14" t="inlineStr"/>
       <c r="L7" s="14" t="inlineStr"/>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>#191</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1849,11 +1904,16 @@
       </c>
       <c r="J8" s="14" t="inlineStr">
         <is>
-          <t>chore/m0-stabilize</t>
+          <t>chore/m0-7</t>
         </is>
       </c>
       <c r="K8" s="14" t="inlineStr"/>
       <c r="L8" s="14" t="inlineStr"/>
+      <c r="M8" s="15" t="inlineStr">
+        <is>
+          <t>#192</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1901,11 +1961,16 @@
       </c>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>chore/m0-stabilize</t>
+          <t>chore/m0-8</t>
         </is>
       </c>
       <c r="K9" s="14" t="inlineStr"/>
       <c r="L9" s="14" t="inlineStr"/>
+      <c r="M9" s="15" t="inlineStr">
+        <is>
+          <t>#193</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -1953,11 +2018,16 @@
       </c>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>chore/m0-stabilize</t>
+          <t>chore/m0-9</t>
         </is>
       </c>
       <c r="K10" s="14" t="inlineStr"/>
       <c r="L10" s="14" t="inlineStr"/>
+      <c r="M10" s="15" t="inlineStr">
+        <is>
+          <t>#194</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -2005,11 +2075,16 @@
       </c>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>chore/m0-stabilize</t>
+          <t>chore/m0-10</t>
         </is>
       </c>
       <c r="K11" s="14" t="inlineStr"/>
       <c r="L11" s="14" t="inlineStr"/>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>#195</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -2057,11 +2132,16 @@
       </c>
       <c r="J12" s="14" t="inlineStr">
         <is>
-          <t>chore/m0-stabilize</t>
+          <t>chore/m0-11</t>
         </is>
       </c>
       <c r="K12" s="14" t="inlineStr"/>
       <c r="L12" s="14" t="inlineStr"/>
+      <c r="M12" s="15" t="inlineStr">
+        <is>
+          <t>#196</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -2109,11 +2189,16 @@
       </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
-          <t>feat/m1-foundation</t>
+          <t>feat/m1-1</t>
         </is>
       </c>
       <c r="K13" s="14" t="inlineStr"/>
       <c r="L13" s="14" t="inlineStr"/>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>#197</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -2161,11 +2246,16 @@
       </c>
       <c r="J14" s="14" t="inlineStr">
         <is>
-          <t>feat/m1-foundation</t>
+          <t>feat/m1-2</t>
         </is>
       </c>
       <c r="K14" s="14" t="inlineStr"/>
       <c r="L14" s="14" t="inlineStr"/>
+      <c r="M14" s="15" t="inlineStr">
+        <is>
+          <t>#198</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -2213,11 +2303,16 @@
       </c>
       <c r="J15" s="14" t="inlineStr">
         <is>
-          <t>feat/m1-foundation</t>
+          <t>feat/m1-3</t>
         </is>
       </c>
       <c r="K15" s="14" t="inlineStr"/>
       <c r="L15" s="14" t="inlineStr"/>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>#199</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -2265,11 +2360,16 @@
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>feat/m1-foundation</t>
+          <t>feat/m1-4</t>
         </is>
       </c>
       <c r="K16" s="14" t="inlineStr"/>
       <c r="L16" s="14" t="inlineStr"/>
+      <c r="M16" s="15" t="inlineStr">
+        <is>
+          <t>#200</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -2317,11 +2417,16 @@
       </c>
       <c r="J17" s="14" t="inlineStr">
         <is>
-          <t>feat/m1-foundation</t>
+          <t>feat/m1-5</t>
         </is>
       </c>
       <c r="K17" s="14" t="inlineStr"/>
       <c r="L17" s="14" t="inlineStr"/>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>#201</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -2369,11 +2474,16 @@
       </c>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>feat/m1-foundation</t>
+          <t>feat/m1-6</t>
         </is>
       </c>
       <c r="K18" s="14" t="inlineStr"/>
       <c r="L18" s="14" t="inlineStr"/>
+      <c r="M18" s="15" t="inlineStr">
+        <is>
+          <t>#202</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -2421,11 +2531,16 @@
       </c>
       <c r="J19" s="14" t="inlineStr">
         <is>
-          <t>feat/m1-foundation</t>
+          <t>feat/m1-7</t>
         </is>
       </c>
       <c r="K19" s="14" t="inlineStr"/>
       <c r="L19" s="14" t="inlineStr"/>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>#203</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -2473,11 +2588,16 @@
       </c>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>feat/m1-foundation</t>
+          <t>feat/m1-8</t>
         </is>
       </c>
       <c r="K20" s="14" t="inlineStr"/>
       <c r="L20" s="14" t="inlineStr"/>
+      <c r="M20" s="15" t="inlineStr">
+        <is>
+          <t>#204</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -2525,11 +2645,16 @@
       </c>
       <c r="J21" s="14" t="inlineStr">
         <is>
-          <t>feat/m1-foundation</t>
+          <t>feat/m1-9</t>
         </is>
       </c>
       <c r="K21" s="14" t="inlineStr"/>
       <c r="L21" s="14" t="inlineStr"/>
+      <c r="M21" s="15" t="inlineStr">
+        <is>
+          <t>#205</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -2577,11 +2702,16 @@
       </c>
       <c r="J22" s="14" t="inlineStr">
         <is>
-          <t>feat/m1-foundation</t>
+          <t>feat/m1-10</t>
         </is>
       </c>
       <c r="K22" s="14" t="inlineStr"/>
       <c r="L22" s="14" t="inlineStr"/>
+      <c r="M22" s="15" t="inlineStr">
+        <is>
+          <t>#206</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -2629,11 +2759,16 @@
       </c>
       <c r="J23" s="14" t="inlineStr">
         <is>
-          <t>feat/m1-foundation</t>
+          <t>feat/m1-11</t>
         </is>
       </c>
       <c r="K23" s="14" t="inlineStr"/>
       <c r="L23" s="14" t="inlineStr"/>
+      <c r="M23" s="15" t="inlineStr">
+        <is>
+          <t>#207</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -2681,11 +2816,16 @@
       </c>
       <c r="J24" s="14" t="inlineStr">
         <is>
-          <t>feat/m1-foundation</t>
+          <t>feat/m1-12</t>
         </is>
       </c>
       <c r="K24" s="14" t="inlineStr"/>
       <c r="L24" s="14" t="inlineStr"/>
+      <c r="M24" s="15" t="inlineStr">
+        <is>
+          <t>#208</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -2733,11 +2873,16 @@
       </c>
       <c r="J25" s="14" t="inlineStr">
         <is>
-          <t>feat/m1-foundation</t>
+          <t>feat/m1-13</t>
         </is>
       </c>
       <c r="K25" s="14" t="inlineStr"/>
       <c r="L25" s="14" t="inlineStr"/>
+      <c r="M25" s="15" t="inlineStr">
+        <is>
+          <t>#209</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -2785,11 +2930,16 @@
       </c>
       <c r="J26" s="14" t="inlineStr">
         <is>
-          <t>feat/m1-foundation</t>
+          <t>feat/m1-14</t>
         </is>
       </c>
       <c r="K26" s="14" t="inlineStr"/>
       <c r="L26" s="14" t="inlineStr"/>
+      <c r="M26" s="15" t="inlineStr">
+        <is>
+          <t>#210</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -2837,11 +2987,16 @@
       </c>
       <c r="J27" s="14" t="inlineStr">
         <is>
-          <t>feat/m2-mikrotik-sync</t>
+          <t>feat/m2-1</t>
         </is>
       </c>
       <c r="K27" s="14" t="inlineStr"/>
       <c r="L27" s="14" t="inlineStr"/>
+      <c r="M27" s="15" t="inlineStr">
+        <is>
+          <t>#211</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -2889,11 +3044,16 @@
       </c>
       <c r="J28" s="14" t="inlineStr">
         <is>
-          <t>feat/m2-mikrotik-sync</t>
+          <t>feat/m2-2</t>
         </is>
       </c>
       <c r="K28" s="14" t="inlineStr"/>
       <c r="L28" s="14" t="inlineStr"/>
+      <c r="M28" s="15" t="inlineStr">
+        <is>
+          <t>#212</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -2941,11 +3101,16 @@
       </c>
       <c r="J29" s="14" t="inlineStr">
         <is>
-          <t>feat/m2-mikrotik-sync</t>
+          <t>feat/m2-3</t>
         </is>
       </c>
       <c r="K29" s="14" t="inlineStr"/>
       <c r="L29" s="14" t="inlineStr"/>
+      <c r="M29" s="15" t="inlineStr">
+        <is>
+          <t>#213</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -2993,11 +3158,16 @@
       </c>
       <c r="J30" s="14" t="inlineStr">
         <is>
-          <t>feat/m2-mikrotik-sync</t>
+          <t>feat/m2-4</t>
         </is>
       </c>
       <c r="K30" s="14" t="inlineStr"/>
       <c r="L30" s="14" t="inlineStr"/>
+      <c r="M30" s="15" t="inlineStr">
+        <is>
+          <t>#214</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -3045,11 +3215,16 @@
       </c>
       <c r="J31" s="14" t="inlineStr">
         <is>
-          <t>feat/m2-mikrotik-sync</t>
+          <t>feat/m2-5</t>
         </is>
       </c>
       <c r="K31" s="14" t="inlineStr"/>
       <c r="L31" s="14" t="inlineStr"/>
+      <c r="M31" s="15" t="inlineStr">
+        <is>
+          <t>#215</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -3097,11 +3272,16 @@
       </c>
       <c r="J32" s="14" t="inlineStr">
         <is>
-          <t>feat/m2-mikrotik-sync</t>
+          <t>feat/m2-6</t>
         </is>
       </c>
       <c r="K32" s="14" t="inlineStr"/>
       <c r="L32" s="14" t="inlineStr"/>
+      <c r="M32" s="15" t="inlineStr">
+        <is>
+          <t>#216</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -3149,11 +3329,16 @@
       </c>
       <c r="J33" s="14" t="inlineStr">
         <is>
-          <t>feat/m2-mikrotik-sync</t>
+          <t>feat/m2-7</t>
         </is>
       </c>
       <c r="K33" s="14" t="inlineStr"/>
       <c r="L33" s="14" t="inlineStr"/>
+      <c r="M33" s="15" t="inlineStr">
+        <is>
+          <t>#217</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -3201,11 +3386,16 @@
       </c>
       <c r="J34" s="14" t="inlineStr">
         <is>
-          <t>feat/m2-mikrotik-sync</t>
+          <t>feat/m2-8</t>
         </is>
       </c>
       <c r="K34" s="14" t="inlineStr"/>
       <c r="L34" s="14" t="inlineStr"/>
+      <c r="M34" s="15" t="inlineStr">
+        <is>
+          <t>#218</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -3253,11 +3443,16 @@
       </c>
       <c r="J35" s="14" t="inlineStr">
         <is>
-          <t>feat/m2-mikrotik-sync</t>
+          <t>feat/m2-9</t>
         </is>
       </c>
       <c r="K35" s="14" t="inlineStr"/>
       <c r="L35" s="14" t="inlineStr"/>
+      <c r="M35" s="15" t="inlineStr">
+        <is>
+          <t>#219</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -3305,11 +3500,16 @@
       </c>
       <c r="J36" s="14" t="inlineStr">
         <is>
-          <t>feat/m2-mikrotik-sync</t>
+          <t>feat/m2-10</t>
         </is>
       </c>
       <c r="K36" s="14" t="inlineStr"/>
       <c r="L36" s="14" t="inlineStr"/>
+      <c r="M36" s="15" t="inlineStr">
+        <is>
+          <t>#220</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -3357,11 +3557,16 @@
       </c>
       <c r="J37" s="14" t="inlineStr">
         <is>
-          <t>feat/m2-mikrotik-sync</t>
+          <t>feat/m2-11</t>
         </is>
       </c>
       <c r="K37" s="14" t="inlineStr"/>
       <c r="L37" s="14" t="inlineStr"/>
+      <c r="M37" s="15" t="inlineStr">
+        <is>
+          <t>#221</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -3409,11 +3614,16 @@
       </c>
       <c r="J38" s="14" t="inlineStr">
         <is>
-          <t>feat/m2-mikrotik-sync</t>
+          <t>feat/m2-12</t>
         </is>
       </c>
       <c r="K38" s="14" t="inlineStr"/>
       <c r="L38" s="14" t="inlineStr"/>
+      <c r="M38" s="15" t="inlineStr">
+        <is>
+          <t>#222</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -3461,11 +3671,16 @@
       </c>
       <c r="J39" s="14" t="inlineStr">
         <is>
-          <t>feat/m2-mikrotik-sync</t>
+          <t>feat/m2-14</t>
         </is>
       </c>
       <c r="K39" s="14" t="inlineStr"/>
       <c r="L39" s="14" t="inlineStr"/>
+      <c r="M39" s="15" t="inlineStr">
+        <is>
+          <t>#223</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -3513,11 +3728,16 @@
       </c>
       <c r="J40" s="14" t="inlineStr">
         <is>
-          <t>feat/m2-mikrotik-sync</t>
+          <t>feat/m2-13</t>
         </is>
       </c>
       <c r="K40" s="14" t="inlineStr"/>
       <c r="L40" s="14" t="inlineStr"/>
+      <c r="M40" s="15" t="inlineStr">
+        <is>
+          <t>#224</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
@@ -3565,11 +3785,16 @@
       </c>
       <c r="J41" s="14" t="inlineStr">
         <is>
-          <t>feat/m3-data-engine</t>
+          <t>feat/m3-1</t>
         </is>
       </c>
       <c r="K41" s="14" t="inlineStr"/>
       <c r="L41" s="14" t="inlineStr"/>
+      <c r="M41" s="15" t="inlineStr">
+        <is>
+          <t>#225</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
@@ -3617,11 +3842,16 @@
       </c>
       <c r="J42" s="14" t="inlineStr">
         <is>
-          <t>feat/m3-data-engine</t>
+          <t>feat/m3-2</t>
         </is>
       </c>
       <c r="K42" s="14" t="inlineStr"/>
       <c r="L42" s="14" t="inlineStr"/>
+      <c r="M42" s="15" t="inlineStr">
+        <is>
+          <t>#226</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
@@ -3669,11 +3899,16 @@
       </c>
       <c r="J43" s="14" t="inlineStr">
         <is>
-          <t>feat/m3-data-engine</t>
+          <t>feat/m3-3</t>
         </is>
       </c>
       <c r="K43" s="14" t="inlineStr"/>
       <c r="L43" s="14" t="inlineStr"/>
+      <c r="M43" s="15" t="inlineStr">
+        <is>
+          <t>#227</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -3721,11 +3956,16 @@
       </c>
       <c r="J44" s="14" t="inlineStr">
         <is>
-          <t>feat/m3-data-engine</t>
+          <t>feat/m3-4</t>
         </is>
       </c>
       <c r="K44" s="14" t="inlineStr"/>
       <c r="L44" s="14" t="inlineStr"/>
+      <c r="M44" s="15" t="inlineStr">
+        <is>
+          <t>#228</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
@@ -3773,11 +4013,16 @@
       </c>
       <c r="J45" s="14" t="inlineStr">
         <is>
-          <t>feat/m3-data-engine</t>
+          <t>feat/m3-5</t>
         </is>
       </c>
       <c r="K45" s="14" t="inlineStr"/>
       <c r="L45" s="14" t="inlineStr"/>
+      <c r="M45" s="15" t="inlineStr">
+        <is>
+          <t>#229</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
@@ -3825,11 +4070,16 @@
       </c>
       <c r="J46" s="14" t="inlineStr">
         <is>
-          <t>feat/m3-data-engine</t>
+          <t>feat/m3-6</t>
         </is>
       </c>
       <c r="K46" s="14" t="inlineStr"/>
       <c r="L46" s="14" t="inlineStr"/>
+      <c r="M46" s="15" t="inlineStr">
+        <is>
+          <t>#230</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
@@ -3877,11 +4127,16 @@
       </c>
       <c r="J47" s="14" t="inlineStr">
         <is>
-          <t>feat/m3-data-engine</t>
+          <t>feat/m3-7</t>
         </is>
       </c>
       <c r="K47" s="14" t="inlineStr"/>
       <c r="L47" s="14" t="inlineStr"/>
+      <c r="M47" s="15" t="inlineStr">
+        <is>
+          <t>#231</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
@@ -3929,11 +4184,16 @@
       </c>
       <c r="J48" s="14" t="inlineStr">
         <is>
-          <t>feat/m3-data-engine</t>
+          <t>feat/m3-8</t>
         </is>
       </c>
       <c r="K48" s="14" t="inlineStr"/>
       <c r="L48" s="14" t="inlineStr"/>
+      <c r="M48" s="15" t="inlineStr">
+        <is>
+          <t>#232</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
@@ -3981,11 +4241,16 @@
       </c>
       <c r="J49" s="14" t="inlineStr">
         <is>
-          <t>feat/m3-data-engine</t>
+          <t>feat/m3-9</t>
         </is>
       </c>
       <c r="K49" s="14" t="inlineStr"/>
       <c r="L49" s="14" t="inlineStr"/>
+      <c r="M49" s="15" t="inlineStr">
+        <is>
+          <t>#233</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
@@ -4033,11 +4298,16 @@
       </c>
       <c r="J50" s="14" t="inlineStr">
         <is>
-          <t>feat/m3-data-engine</t>
+          <t>feat/m3-10</t>
         </is>
       </c>
       <c r="K50" s="14" t="inlineStr"/>
       <c r="L50" s="14" t="inlineStr"/>
+      <c r="M50" s="15" t="inlineStr">
+        <is>
+          <t>#234</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
@@ -4085,11 +4355,16 @@
       </c>
       <c r="J51" s="14" t="inlineStr">
         <is>
-          <t>feat/m3-data-engine</t>
+          <t>feat/m3-11</t>
         </is>
       </c>
       <c r="K51" s="14" t="inlineStr"/>
       <c r="L51" s="14" t="inlineStr"/>
+      <c r="M51" s="15" t="inlineStr">
+        <is>
+          <t>#235</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
@@ -4137,11 +4412,16 @@
       </c>
       <c r="J52" s="14" t="inlineStr">
         <is>
-          <t>feat/m3-data-engine</t>
+          <t>feat/m3-12</t>
         </is>
       </c>
       <c r="K52" s="14" t="inlineStr"/>
       <c r="L52" s="14" t="inlineStr"/>
+      <c r="M52" s="15" t="inlineStr">
+        <is>
+          <t>#236</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
@@ -4189,11 +4469,16 @@
       </c>
       <c r="J53" s="14" t="inlineStr">
         <is>
-          <t>feat/m4-owner-ops</t>
+          <t>feat/m4-1</t>
         </is>
       </c>
       <c r="K53" s="14" t="inlineStr"/>
       <c r="L53" s="14" t="inlineStr"/>
+      <c r="M53" s="15" t="inlineStr">
+        <is>
+          <t>#237</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
@@ -4241,11 +4526,16 @@
       </c>
       <c r="J54" s="14" t="inlineStr">
         <is>
-          <t>feat/m4-owner-ops</t>
+          <t>feat/m4-2</t>
         </is>
       </c>
       <c r="K54" s="14" t="inlineStr"/>
       <c r="L54" s="14" t="inlineStr"/>
+      <c r="M54" s="15" t="inlineStr">
+        <is>
+          <t>#238</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
@@ -4293,11 +4583,16 @@
       </c>
       <c r="J55" s="14" t="inlineStr">
         <is>
-          <t>feat/m4-owner-ops</t>
+          <t>feat/m4-3</t>
         </is>
       </c>
       <c r="K55" s="14" t="inlineStr"/>
       <c r="L55" s="14" t="inlineStr"/>
+      <c r="M55" s="15" t="inlineStr">
+        <is>
+          <t>#239</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
@@ -4345,11 +4640,16 @@
       </c>
       <c r="J56" s="14" t="inlineStr">
         <is>
-          <t>feat/m4-owner-ops</t>
+          <t>feat/m4-4</t>
         </is>
       </c>
       <c r="K56" s="14" t="inlineStr"/>
       <c r="L56" s="14" t="inlineStr"/>
+      <c r="M56" s="15" t="inlineStr">
+        <is>
+          <t>#240</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
@@ -4397,11 +4697,16 @@
       </c>
       <c r="J57" s="14" t="inlineStr">
         <is>
-          <t>feat/m4-owner-ops</t>
+          <t>feat/m4-5</t>
         </is>
       </c>
       <c r="K57" s="14" t="inlineStr"/>
       <c r="L57" s="14" t="inlineStr"/>
+      <c r="M57" s="15" t="inlineStr">
+        <is>
+          <t>#241</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
@@ -4449,11 +4754,16 @@
       </c>
       <c r="J58" s="14" t="inlineStr">
         <is>
-          <t>feat/m4-owner-ops</t>
+          <t>feat/m4-6</t>
         </is>
       </c>
       <c r="K58" s="14" t="inlineStr"/>
       <c r="L58" s="14" t="inlineStr"/>
+      <c r="M58" s="15" t="inlineStr">
+        <is>
+          <t>#242</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
@@ -4501,11 +4811,16 @@
       </c>
       <c r="J59" s="14" t="inlineStr">
         <is>
-          <t>feat/m4-owner-ops</t>
+          <t>feat/m4-7</t>
         </is>
       </c>
       <c r="K59" s="14" t="inlineStr"/>
       <c r="L59" s="14" t="inlineStr"/>
+      <c r="M59" s="15" t="inlineStr">
+        <is>
+          <t>#243</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
@@ -4553,11 +4868,16 @@
       </c>
       <c r="J60" s="14" t="inlineStr">
         <is>
-          <t>feat/m4-owner-ops</t>
+          <t>feat/m4-8</t>
         </is>
       </c>
       <c r="K60" s="14" t="inlineStr"/>
       <c r="L60" s="14" t="inlineStr"/>
+      <c r="M60" s="15" t="inlineStr">
+        <is>
+          <t>#244</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
@@ -4605,11 +4925,16 @@
       </c>
       <c r="J61" s="14" t="inlineStr">
         <is>
-          <t>feat/m4-owner-ops</t>
+          <t>feat/m4-9</t>
         </is>
       </c>
       <c r="K61" s="14" t="inlineStr"/>
       <c r="L61" s="14" t="inlineStr"/>
+      <c r="M61" s="15" t="inlineStr">
+        <is>
+          <t>#245</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
@@ -4657,11 +4982,16 @@
       </c>
       <c r="J62" s="14" t="inlineStr">
         <is>
-          <t>feat/m4-owner-ops</t>
+          <t>feat/m4-10</t>
         </is>
       </c>
       <c r="K62" s="14" t="inlineStr"/>
       <c r="L62" s="14" t="inlineStr"/>
+      <c r="M62" s="15" t="inlineStr">
+        <is>
+          <t>#246</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
@@ -4709,11 +5039,16 @@
       </c>
       <c r="J63" s="14" t="inlineStr">
         <is>
-          <t>feat/m4-owner-ops</t>
+          <t>feat/m4-11</t>
         </is>
       </c>
       <c r="K63" s="14" t="inlineStr"/>
       <c r="L63" s="14" t="inlineStr"/>
+      <c r="M63" s="15" t="inlineStr">
+        <is>
+          <t>#247</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
@@ -4761,11 +5096,16 @@
       </c>
       <c r="J64" s="14" t="inlineStr">
         <is>
-          <t>feat/m4-owner-ops</t>
+          <t>feat/m4-12</t>
         </is>
       </c>
       <c r="K64" s="14" t="inlineStr"/>
       <c r="L64" s="14" t="inlineStr"/>
+      <c r="M64" s="15" t="inlineStr">
+        <is>
+          <t>#248</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
@@ -4813,11 +5153,16 @@
       </c>
       <c r="J65" s="14" t="inlineStr">
         <is>
-          <t>feat/m4-owner-ops</t>
+          <t>feat/m4-13</t>
         </is>
       </c>
       <c r="K65" s="14" t="inlineStr"/>
       <c r="L65" s="14" t="inlineStr"/>
+      <c r="M65" s="15" t="inlineStr">
+        <is>
+          <t>#249</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
@@ -4865,11 +5210,16 @@
       </c>
       <c r="J66" s="14" t="inlineStr">
         <is>
-          <t>feat/m4-owner-ops</t>
+          <t>feat/m4-14</t>
         </is>
       </c>
       <c r="K66" s="14" t="inlineStr"/>
       <c r="L66" s="14" t="inlineStr"/>
+      <c r="M66" s="15" t="inlineStr">
+        <is>
+          <t>#250</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
@@ -4917,11 +5267,16 @@
       </c>
       <c r="J67" s="14" t="inlineStr">
         <is>
-          <t>feat/m4-owner-ops</t>
+          <t>feat/m4-15</t>
         </is>
       </c>
       <c r="K67" s="14" t="inlineStr"/>
       <c r="L67" s="14" t="inlineStr"/>
+      <c r="M67" s="15" t="inlineStr">
+        <is>
+          <t>#251</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
@@ -4969,11 +5324,16 @@
       </c>
       <c r="J68" s="14" t="inlineStr">
         <is>
-          <t>feat/m4-owner-ops</t>
+          <t>feat/m4-16</t>
         </is>
       </c>
       <c r="K68" s="14" t="inlineStr"/>
       <c r="L68" s="14" t="inlineStr"/>
+      <c r="M68" s="15" t="inlineStr">
+        <is>
+          <t>#252</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
@@ -5021,11 +5381,16 @@
       </c>
       <c r="J69" s="14" t="inlineStr">
         <is>
-          <t>feat/m4-owner-ops</t>
+          <t>feat/m4-17</t>
         </is>
       </c>
       <c r="K69" s="14" t="inlineStr"/>
       <c r="L69" s="14" t="inlineStr"/>
+      <c r="M69" s="15" t="inlineStr">
+        <is>
+          <t>#253</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
@@ -5073,11 +5438,16 @@
       </c>
       <c r="J70" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-1</t>
         </is>
       </c>
       <c r="K70" s="14" t="inlineStr"/>
       <c r="L70" s="14" t="inlineStr"/>
+      <c r="M70" s="15" t="inlineStr">
+        <is>
+          <t>#254</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
@@ -5125,11 +5495,16 @@
       </c>
       <c r="J71" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-2</t>
         </is>
       </c>
       <c r="K71" s="14" t="inlineStr"/>
       <c r="L71" s="14" t="inlineStr"/>
+      <c r="M71" s="15" t="inlineStr">
+        <is>
+          <t>#255</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
@@ -5177,11 +5552,16 @@
       </c>
       <c r="J72" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-3</t>
         </is>
       </c>
       <c r="K72" s="14" t="inlineStr"/>
       <c r="L72" s="14" t="inlineStr"/>
+      <c r="M72" s="15" t="inlineStr">
+        <is>
+          <t>#256</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
@@ -5229,11 +5609,16 @@
       </c>
       <c r="J73" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-4</t>
         </is>
       </c>
       <c r="K73" s="14" t="inlineStr"/>
       <c r="L73" s="14" t="inlineStr"/>
+      <c r="M73" s="15" t="inlineStr">
+        <is>
+          <t>#257</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
@@ -5281,11 +5666,16 @@
       </c>
       <c r="J74" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-5</t>
         </is>
       </c>
       <c r="K74" s="14" t="inlineStr"/>
       <c r="L74" s="14" t="inlineStr"/>
+      <c r="M74" s="15" t="inlineStr">
+        <is>
+          <t>#258</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
@@ -5333,11 +5723,16 @@
       </c>
       <c r="J75" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-6</t>
         </is>
       </c>
       <c r="K75" s="14" t="inlineStr"/>
       <c r="L75" s="14" t="inlineStr"/>
+      <c r="M75" s="15" t="inlineStr">
+        <is>
+          <t>#259</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
@@ -5385,11 +5780,16 @@
       </c>
       <c r="J76" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-7</t>
         </is>
       </c>
       <c r="K76" s="14" t="inlineStr"/>
       <c r="L76" s="14" t="inlineStr"/>
+      <c r="M76" s="15" t="inlineStr">
+        <is>
+          <t>#260</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
@@ -5437,11 +5837,16 @@
       </c>
       <c r="J77" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-8</t>
         </is>
       </c>
       <c r="K77" s="14" t="inlineStr"/>
       <c r="L77" s="14" t="inlineStr"/>
+      <c r="M77" s="15" t="inlineStr">
+        <is>
+          <t>#261</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
@@ -5489,11 +5894,16 @@
       </c>
       <c r="J78" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-9</t>
         </is>
       </c>
       <c r="K78" s="14" t="inlineStr"/>
       <c r="L78" s="14" t="inlineStr"/>
+      <c r="M78" s="15" t="inlineStr">
+        <is>
+          <t>#262</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
@@ -5541,11 +5951,16 @@
       </c>
       <c r="J79" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-10</t>
         </is>
       </c>
       <c r="K79" s="14" t="inlineStr"/>
       <c r="L79" s="14" t="inlineStr"/>
+      <c r="M79" s="15" t="inlineStr">
+        <is>
+          <t>#263</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
@@ -5593,11 +6008,16 @@
       </c>
       <c r="J80" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-11</t>
         </is>
       </c>
       <c r="K80" s="14" t="inlineStr"/>
       <c r="L80" s="14" t="inlineStr"/>
+      <c r="M80" s="15" t="inlineStr">
+        <is>
+          <t>#264</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
@@ -5645,11 +6065,16 @@
       </c>
       <c r="J81" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-12</t>
         </is>
       </c>
       <c r="K81" s="14" t="inlineStr"/>
       <c r="L81" s="14" t="inlineStr"/>
+      <c r="M81" s="15" t="inlineStr">
+        <is>
+          <t>#265</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
@@ -5697,11 +6122,16 @@
       </c>
       <c r="J82" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-13</t>
         </is>
       </c>
       <c r="K82" s="14" t="inlineStr"/>
       <c r="L82" s="14" t="inlineStr"/>
+      <c r="M82" s="15" t="inlineStr">
+        <is>
+          <t>#266</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
@@ -5749,11 +6179,16 @@
       </c>
       <c r="J83" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-14</t>
         </is>
       </c>
       <c r="K83" s="14" t="inlineStr"/>
       <c r="L83" s="14" t="inlineStr"/>
+      <c r="M83" s="15" t="inlineStr">
+        <is>
+          <t>#267</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
@@ -5801,11 +6236,16 @@
       </c>
       <c r="J84" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-15</t>
         </is>
       </c>
       <c r="K84" s="14" t="inlineStr"/>
       <c r="L84" s="14" t="inlineStr"/>
+      <c r="M84" s="15" t="inlineStr">
+        <is>
+          <t>#268</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
@@ -5853,11 +6293,16 @@
       </c>
       <c r="J85" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-16</t>
         </is>
       </c>
       <c r="K85" s="14" t="inlineStr"/>
       <c r="L85" s="14" t="inlineStr"/>
+      <c r="M85" s="15" t="inlineStr">
+        <is>
+          <t>#269</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
@@ -5905,11 +6350,16 @@
       </c>
       <c r="J86" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-17</t>
         </is>
       </c>
       <c r="K86" s="14" t="inlineStr"/>
       <c r="L86" s="14" t="inlineStr"/>
+      <c r="M86" s="15" t="inlineStr">
+        <is>
+          <t>#270</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
@@ -5957,11 +6407,16 @@
       </c>
       <c r="J87" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-18</t>
         </is>
       </c>
       <c r="K87" s="14" t="inlineStr"/>
       <c r="L87" s="14" t="inlineStr"/>
+      <c r="M87" s="15" t="inlineStr">
+        <is>
+          <t>#271</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
@@ -6009,11 +6464,16 @@
       </c>
       <c r="J88" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-19</t>
         </is>
       </c>
       <c r="K88" s="14" t="inlineStr"/>
       <c r="L88" s="14" t="inlineStr"/>
+      <c r="M88" s="15" t="inlineStr">
+        <is>
+          <t>#272</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
@@ -6061,11 +6521,16 @@
       </c>
       <c r="J89" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-20</t>
         </is>
       </c>
       <c r="K89" s="14" t="inlineStr"/>
       <c r="L89" s="14" t="inlineStr"/>
+      <c r="M89" s="15" t="inlineStr">
+        <is>
+          <t>#273</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
@@ -6113,11 +6578,16 @@
       </c>
       <c r="J90" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-21</t>
         </is>
       </c>
       <c r="K90" s="14" t="inlineStr"/>
       <c r="L90" s="14" t="inlineStr"/>
+      <c r="M90" s="15" t="inlineStr">
+        <is>
+          <t>#274</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
@@ -6165,11 +6635,16 @@
       </c>
       <c r="J91" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-22</t>
         </is>
       </c>
       <c r="K91" s="14" t="inlineStr"/>
       <c r="L91" s="14" t="inlineStr"/>
+      <c r="M91" s="15" t="inlineStr">
+        <is>
+          <t>#275</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
@@ -6217,11 +6692,16 @@
       </c>
       <c r="J92" s="14" t="inlineStr">
         <is>
-          <t>feat/m5-finance-v2</t>
+          <t>feat/m5-23</t>
         </is>
       </c>
       <c r="K92" s="14" t="inlineStr"/>
       <c r="L92" s="14" t="inlineStr"/>
+      <c r="M92" s="15" t="inlineStr">
+        <is>
+          <t>#276</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
@@ -6269,11 +6749,16 @@
       </c>
       <c r="J93" s="14" t="inlineStr">
         <is>
-          <t>feat/m6-gsg-ur</t>
+          <t>feat/m6-1</t>
         </is>
       </c>
       <c r="K93" s="14" t="inlineStr"/>
       <c r="L93" s="14" t="inlineStr"/>
+      <c r="M93" s="15" t="inlineStr">
+        <is>
+          <t>#277</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
@@ -6321,11 +6806,16 @@
       </c>
       <c r="J94" s="14" t="inlineStr">
         <is>
-          <t>feat/m6-gsg-ur</t>
+          <t>feat/m6-2</t>
         </is>
       </c>
       <c r="K94" s="14" t="inlineStr"/>
       <c r="L94" s="14" t="inlineStr"/>
+      <c r="M94" s="15" t="inlineStr">
+        <is>
+          <t>#278</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
@@ -6373,11 +6863,16 @@
       </c>
       <c r="J95" s="14" t="inlineStr">
         <is>
-          <t>feat/m6-gsg-ur</t>
+          <t>feat/m6-3</t>
         </is>
       </c>
       <c r="K95" s="14" t="inlineStr"/>
       <c r="L95" s="14" t="inlineStr"/>
+      <c r="M95" s="15" t="inlineStr">
+        <is>
+          <t>#279</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
@@ -6425,11 +6920,16 @@
       </c>
       <c r="J96" s="14" t="inlineStr">
         <is>
-          <t>feat/m6-gsg-ur</t>
+          <t>feat/m6-4</t>
         </is>
       </c>
       <c r="K96" s="14" t="inlineStr"/>
       <c r="L96" s="14" t="inlineStr"/>
+      <c r="M96" s="15" t="inlineStr">
+        <is>
+          <t>#280</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
@@ -6477,11 +6977,16 @@
       </c>
       <c r="J97" s="14" t="inlineStr">
         <is>
-          <t>feat/m6-gsg-ur</t>
+          <t>feat/m6-5</t>
         </is>
       </c>
       <c r="K97" s="14" t="inlineStr"/>
       <c r="L97" s="14" t="inlineStr"/>
+      <c r="M97" s="15" t="inlineStr">
+        <is>
+          <t>#281</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
@@ -6529,11 +7034,16 @@
       </c>
       <c r="J98" s="14" t="inlineStr">
         <is>
-          <t>feat/m6-gsg-ur</t>
+          <t>feat/m6-6</t>
         </is>
       </c>
       <c r="K98" s="14" t="inlineStr"/>
       <c r="L98" s="14" t="inlineStr"/>
+      <c r="M98" s="15" t="inlineStr">
+        <is>
+          <t>#282</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
@@ -6581,11 +7091,16 @@
       </c>
       <c r="J99" s="14" t="inlineStr">
         <is>
-          <t>feat/m6-gsg-ur</t>
+          <t>feat/m6-7</t>
         </is>
       </c>
       <c r="K99" s="14" t="inlineStr"/>
       <c r="L99" s="14" t="inlineStr"/>
+      <c r="M99" s="15" t="inlineStr">
+        <is>
+          <t>#283</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
@@ -6633,11 +7148,16 @@
       </c>
       <c r="J100" s="14" t="inlineStr">
         <is>
-          <t>feat/m6-gsg-ur</t>
+          <t>feat/m6-8</t>
         </is>
       </c>
       <c r="K100" s="14" t="inlineStr"/>
       <c r="L100" s="14" t="inlineStr"/>
+      <c r="M100" s="15" t="inlineStr">
+        <is>
+          <t>#284</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
@@ -6685,11 +7205,16 @@
       </c>
       <c r="J101" s="14" t="inlineStr">
         <is>
-          <t>feat/m6-gsg-ur</t>
+          <t>feat/m6-9</t>
         </is>
       </c>
       <c r="K101" s="14" t="inlineStr"/>
       <c r="L101" s="14" t="inlineStr"/>
+      <c r="M101" s="15" t="inlineStr">
+        <is>
+          <t>#285</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
@@ -6737,11 +7262,16 @@
       </c>
       <c r="J102" s="14" t="inlineStr">
         <is>
-          <t>feat/m6-gsg-ur</t>
+          <t>feat/m6-14</t>
         </is>
       </c>
       <c r="K102" s="14" t="inlineStr"/>
       <c r="L102" s="14" t="inlineStr"/>
+      <c r="M102" s="15" t="inlineStr">
+        <is>
+          <t>#286</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
@@ -6789,11 +7319,16 @@
       </c>
       <c r="J103" s="14" t="inlineStr">
         <is>
-          <t>feat/m6-gsg-ur</t>
+          <t>feat/m6-10</t>
         </is>
       </c>
       <c r="K103" s="14" t="inlineStr"/>
       <c r="L103" s="14" t="inlineStr"/>
+      <c r="M103" s="15" t="inlineStr">
+        <is>
+          <t>#287</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
@@ -6841,11 +7376,16 @@
       </c>
       <c r="J104" s="14" t="inlineStr">
         <is>
-          <t>feat/m6-gsg-ur</t>
+          <t>feat/m6-11</t>
         </is>
       </c>
       <c r="K104" s="14" t="inlineStr"/>
       <c r="L104" s="14" t="inlineStr"/>
+      <c r="M104" s="15" t="inlineStr">
+        <is>
+          <t>#288</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
@@ -6893,11 +7433,16 @@
       </c>
       <c r="J105" s="14" t="inlineStr">
         <is>
-          <t>feat/m6-gsg-ur</t>
+          <t>feat/m6-12</t>
         </is>
       </c>
       <c r="K105" s="14" t="inlineStr"/>
       <c r="L105" s="14" t="inlineStr"/>
+      <c r="M105" s="15" t="inlineStr">
+        <is>
+          <t>#289</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
@@ -6945,11 +7490,16 @@
       </c>
       <c r="J106" s="14" t="inlineStr">
         <is>
-          <t>feat/m6-gsg-ur</t>
+          <t>feat/m6-13</t>
         </is>
       </c>
       <c r="K106" s="14" t="inlineStr"/>
       <c r="L106" s="14" t="inlineStr"/>
+      <c r="M106" s="15" t="inlineStr">
+        <is>
+          <t>#290</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
@@ -6997,11 +7547,16 @@
       </c>
       <c r="J107" s="14" t="inlineStr">
         <is>
-          <t>feat/m7-reports</t>
+          <t>feat/m7-1</t>
         </is>
       </c>
       <c r="K107" s="14" t="inlineStr"/>
       <c r="L107" s="14" t="inlineStr"/>
+      <c r="M107" s="15" t="inlineStr">
+        <is>
+          <t>#291</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
@@ -7049,11 +7604,16 @@
       </c>
       <c r="J108" s="14" t="inlineStr">
         <is>
-          <t>feat/m7-reports</t>
+          <t>feat/m7-2</t>
         </is>
       </c>
       <c r="K108" s="14" t="inlineStr"/>
       <c r="L108" s="14" t="inlineStr"/>
+      <c r="M108" s="15" t="inlineStr">
+        <is>
+          <t>#292</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
@@ -7101,11 +7661,16 @@
       </c>
       <c r="J109" s="14" t="inlineStr">
         <is>
-          <t>feat/m7-reports</t>
+          <t>feat/m7-3</t>
         </is>
       </c>
       <c r="K109" s="14" t="inlineStr"/>
       <c r="L109" s="14" t="inlineStr"/>
+      <c r="M109" s="15" t="inlineStr">
+        <is>
+          <t>#293</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
@@ -7153,11 +7718,16 @@
       </c>
       <c r="J110" s="14" t="inlineStr">
         <is>
-          <t>feat/m7-reports</t>
+          <t>feat/m7-4</t>
         </is>
       </c>
       <c r="K110" s="14" t="inlineStr"/>
       <c r="L110" s="14" t="inlineStr"/>
+      <c r="M110" s="15" t="inlineStr">
+        <is>
+          <t>#294</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
@@ -7205,11 +7775,16 @@
       </c>
       <c r="J111" s="14" t="inlineStr">
         <is>
-          <t>feat/m7-reports</t>
+          <t>feat/m7-5</t>
         </is>
       </c>
       <c r="K111" s="14" t="inlineStr"/>
       <c r="L111" s="14" t="inlineStr"/>
+      <c r="M111" s="15" t="inlineStr">
+        <is>
+          <t>#295</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
@@ -7257,11 +7832,16 @@
       </c>
       <c r="J112" s="14" t="inlineStr">
         <is>
-          <t>feat/m8-super-admin</t>
+          <t>feat/m8-1</t>
         </is>
       </c>
       <c r="K112" s="14" t="inlineStr"/>
       <c r="L112" s="14" t="inlineStr"/>
+      <c r="M112" s="15" t="inlineStr">
+        <is>
+          <t>#296</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
@@ -7309,11 +7889,16 @@
       </c>
       <c r="J113" s="14" t="inlineStr">
         <is>
-          <t>feat/m8-super-admin</t>
+          <t>feat/m8-2</t>
         </is>
       </c>
       <c r="K113" s="14" t="inlineStr"/>
       <c r="L113" s="14" t="inlineStr"/>
+      <c r="M113" s="15" t="inlineStr">
+        <is>
+          <t>#297</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="5" t="inlineStr">
@@ -7361,11 +7946,16 @@
       </c>
       <c r="J114" s="14" t="inlineStr">
         <is>
-          <t>feat/m8-super-admin</t>
+          <t>feat/m8-3</t>
         </is>
       </c>
       <c r="K114" s="14" t="inlineStr"/>
       <c r="L114" s="14" t="inlineStr"/>
+      <c r="M114" s="15" t="inlineStr">
+        <is>
+          <t>#298</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="5" t="inlineStr">
@@ -7413,11 +8003,16 @@
       </c>
       <c r="J115" s="14" t="inlineStr">
         <is>
-          <t>feat/m8-super-admin</t>
+          <t>feat/m8-4</t>
         </is>
       </c>
       <c r="K115" s="14" t="inlineStr"/>
       <c r="L115" s="14" t="inlineStr"/>
+      <c r="M115" s="15" t="inlineStr">
+        <is>
+          <t>#299</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="5" t="inlineStr">
@@ -7465,11 +8060,16 @@
       </c>
       <c r="J116" s="14" t="inlineStr">
         <is>
-          <t>feat/m8-super-admin</t>
+          <t>feat/m8-5</t>
         </is>
       </c>
       <c r="K116" s="14" t="inlineStr"/>
       <c r="L116" s="14" t="inlineStr"/>
+      <c r="M116" s="15" t="inlineStr">
+        <is>
+          <t>#300</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
@@ -7517,11 +8117,16 @@
       </c>
       <c r="J117" s="14" t="inlineStr">
         <is>
-          <t>feat/m8-super-admin</t>
+          <t>feat/m8-6</t>
         </is>
       </c>
       <c r="K117" s="14" t="inlineStr"/>
       <c r="L117" s="14" t="inlineStr"/>
+      <c r="M117" s="15" t="inlineStr">
+        <is>
+          <t>#301</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
@@ -7569,11 +8174,16 @@
       </c>
       <c r="J118" s="14" t="inlineStr">
         <is>
-          <t>feat/m8-super-admin</t>
+          <t>feat/m8-7</t>
         </is>
       </c>
       <c r="K118" s="14" t="inlineStr"/>
       <c r="L118" s="14" t="inlineStr"/>
+      <c r="M118" s="15" t="inlineStr">
+        <is>
+          <t>#302</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="5" t="inlineStr">
@@ -7621,11 +8231,16 @@
       </c>
       <c r="J119" s="14" t="inlineStr">
         <is>
-          <t>feat/m8-super-admin</t>
+          <t>feat/m8-8</t>
         </is>
       </c>
       <c r="K119" s="14" t="inlineStr"/>
       <c r="L119" s="14" t="inlineStr"/>
+      <c r="M119" s="15" t="inlineStr">
+        <is>
+          <t>#303</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
@@ -7673,11 +8288,16 @@
       </c>
       <c r="J120" s="14" t="inlineStr">
         <is>
-          <t>feat/m8-super-admin</t>
+          <t>feat/m8-9</t>
         </is>
       </c>
       <c r="K120" s="14" t="inlineStr"/>
       <c r="L120" s="14" t="inlineStr"/>
+      <c r="M120" s="15" t="inlineStr">
+        <is>
+          <t>#304</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
@@ -7725,11 +8345,16 @@
       </c>
       <c r="J121" s="14" t="inlineStr">
         <is>
-          <t>feat/m8-super-admin</t>
+          <t>feat/m8-10</t>
         </is>
       </c>
       <c r="K121" s="14" t="inlineStr"/>
       <c r="L121" s="14" t="inlineStr"/>
+      <c r="M121" s="15" t="inlineStr">
+        <is>
+          <t>#305</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="5" t="inlineStr">
@@ -7777,11 +8402,16 @@
       </c>
       <c r="J122" s="14" t="inlineStr">
         <is>
-          <t>feat/m9-freelancer-portal</t>
+          <t>feat/m9-1</t>
         </is>
       </c>
       <c r="K122" s="14" t="inlineStr"/>
       <c r="L122" s="14" t="inlineStr"/>
+      <c r="M122" s="15" t="inlineStr">
+        <is>
+          <t>#306</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
@@ -7829,11 +8459,16 @@
       </c>
       <c r="J123" s="14" t="inlineStr">
         <is>
-          <t>feat/m9-freelancer-portal</t>
+          <t>feat/m9-2</t>
         </is>
       </c>
       <c r="K123" s="14" t="inlineStr"/>
       <c r="L123" s="14" t="inlineStr"/>
+      <c r="M123" s="15" t="inlineStr">
+        <is>
+          <t>#307</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
@@ -7881,11 +8516,16 @@
       </c>
       <c r="J124" s="14" t="inlineStr">
         <is>
-          <t>feat/m9-freelancer-portal</t>
+          <t>feat/m9-3</t>
         </is>
       </c>
       <c r="K124" s="14" t="inlineStr"/>
       <c r="L124" s="14" t="inlineStr"/>
+      <c r="M124" s="15" t="inlineStr">
+        <is>
+          <t>#308</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="5" t="inlineStr">
@@ -7933,11 +8573,16 @@
       </c>
       <c r="J125" s="14" t="inlineStr">
         <is>
-          <t>feat/m9-freelancer-portal</t>
+          <t>feat/m9-4</t>
         </is>
       </c>
       <c r="K125" s="14" t="inlineStr"/>
       <c r="L125" s="14" t="inlineStr"/>
+      <c r="M125" s="15" t="inlineStr">
+        <is>
+          <t>#309</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="5" t="inlineStr">
@@ -7985,11 +8630,16 @@
       </c>
       <c r="J126" s="14" t="inlineStr">
         <is>
-          <t>feat/m9-freelancer-portal</t>
+          <t>feat/m9-5</t>
         </is>
       </c>
       <c r="K126" s="14" t="inlineStr"/>
       <c r="L126" s="14" t="inlineStr"/>
+      <c r="M126" s="15" t="inlineStr">
+        <is>
+          <t>#310</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="5" t="inlineStr">
@@ -8037,11 +8687,16 @@
       </c>
       <c r="J127" s="14" t="inlineStr">
         <is>
-          <t>feat/m9-freelancer-portal</t>
+          <t>feat/m9-6</t>
         </is>
       </c>
       <c r="K127" s="14" t="inlineStr"/>
       <c r="L127" s="14" t="inlineStr"/>
+      <c r="M127" s="15" t="inlineStr">
+        <is>
+          <t>#311</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="5" t="inlineStr">
@@ -8089,11 +8744,16 @@
       </c>
       <c r="J128" s="14" t="inlineStr">
         <is>
-          <t>feat/m9-freelancer-portal</t>
+          <t>feat/m9-7</t>
         </is>
       </c>
       <c r="K128" s="14" t="inlineStr"/>
       <c r="L128" s="14" t="inlineStr"/>
+      <c r="M128" s="15" t="inlineStr">
+        <is>
+          <t>#312</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="5" t="inlineStr">
@@ -8141,11 +8801,16 @@
       </c>
       <c r="J129" s="14" t="inlineStr">
         <is>
-          <t>feat/m9-freelancer-portal</t>
+          <t>feat/m9-8</t>
         </is>
       </c>
       <c r="K129" s="14" t="inlineStr"/>
       <c r="L129" s="14" t="inlineStr"/>
+      <c r="M129" s="15" t="inlineStr">
+        <is>
+          <t>#313</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="5" t="inlineStr">
@@ -8193,11 +8858,16 @@
       </c>
       <c r="J130" s="14" t="inlineStr">
         <is>
-          <t>feat/m9-freelancer-portal</t>
+          <t>feat/m9-9</t>
         </is>
       </c>
       <c r="K130" s="14" t="inlineStr"/>
       <c r="L130" s="14" t="inlineStr"/>
+      <c r="M130" s="15" t="inlineStr">
+        <is>
+          <t>#314</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="5" t="inlineStr">
@@ -8245,11 +8915,16 @@
       </c>
       <c r="J131" s="14" t="inlineStr">
         <is>
-          <t>feat/m9-freelancer-portal</t>
+          <t>feat/m9-10</t>
         </is>
       </c>
       <c r="K131" s="14" t="inlineStr"/>
       <c r="L131" s="14" t="inlineStr"/>
+      <c r="M131" s="15" t="inlineStr">
+        <is>
+          <t>#315</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="5" t="inlineStr">
@@ -8297,11 +8972,16 @@
       </c>
       <c r="J132" s="14" t="inlineStr">
         <is>
-          <t>feat/m10-public-site</t>
+          <t>feat/m10-1</t>
         </is>
       </c>
       <c r="K132" s="14" t="inlineStr"/>
       <c r="L132" s="14" t="inlineStr"/>
+      <c r="M132" s="15" t="inlineStr">
+        <is>
+          <t>#316</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="5" t="inlineStr">
@@ -8349,11 +9029,16 @@
       </c>
       <c r="J133" s="14" t="inlineStr">
         <is>
-          <t>feat/m10-public-site</t>
+          <t>feat/m10-2</t>
         </is>
       </c>
       <c r="K133" s="14" t="inlineStr"/>
       <c r="L133" s="14" t="inlineStr"/>
+      <c r="M133" s="15" t="inlineStr">
+        <is>
+          <t>#317</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="5" t="inlineStr">
@@ -8401,11 +9086,16 @@
       </c>
       <c r="J134" s="14" t="inlineStr">
         <is>
-          <t>feat/m10-public-site</t>
+          <t>feat/m10-3</t>
         </is>
       </c>
       <c r="K134" s="14" t="inlineStr"/>
       <c r="L134" s="14" t="inlineStr"/>
+      <c r="M134" s="15" t="inlineStr">
+        <is>
+          <t>#318</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="5" t="inlineStr">
@@ -8453,11 +9143,16 @@
       </c>
       <c r="J135" s="14" t="inlineStr">
         <is>
-          <t>feat/m10-public-site</t>
+          <t>feat/m10-4</t>
         </is>
       </c>
       <c r="K135" s="14" t="inlineStr"/>
       <c r="L135" s="14" t="inlineStr"/>
+      <c r="M135" s="15" t="inlineStr">
+        <is>
+          <t>#319</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="5" t="inlineStr">
@@ -8505,11 +9200,16 @@
       </c>
       <c r="J136" s="14" t="inlineStr">
         <is>
-          <t>feat/m10-public-site</t>
+          <t>feat/m10-5</t>
         </is>
       </c>
       <c r="K136" s="14" t="inlineStr"/>
       <c r="L136" s="14" t="inlineStr"/>
+      <c r="M136" s="15" t="inlineStr">
+        <is>
+          <t>#320</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="5" t="inlineStr">
@@ -8557,11 +9257,16 @@
       </c>
       <c r="J137" s="14" t="inlineStr">
         <is>
-          <t>feat/m10-public-site</t>
+          <t>feat/m10-6</t>
         </is>
       </c>
       <c r="K137" s="14" t="inlineStr"/>
       <c r="L137" s="14" t="inlineStr"/>
+      <c r="M137" s="15" t="inlineStr">
+        <is>
+          <t>#321</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="5" t="inlineStr">
@@ -8609,11 +9314,16 @@
       </c>
       <c r="J138" s="14" t="inlineStr">
         <is>
-          <t>feat/m10-public-site</t>
+          <t>feat/m10-7</t>
         </is>
       </c>
       <c r="K138" s="14" t="inlineStr"/>
       <c r="L138" s="14" t="inlineStr"/>
+      <c r="M138" s="15" t="inlineStr">
+        <is>
+          <t>#322</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="5" t="inlineStr">
@@ -8661,11 +9371,16 @@
       </c>
       <c r="J139" s="14" t="inlineStr">
         <is>
-          <t>feat/m10-public-site</t>
+          <t>feat/m10-8</t>
         </is>
       </c>
       <c r="K139" s="14" t="inlineStr"/>
       <c r="L139" s="14" t="inlineStr"/>
+      <c r="M139" s="15" t="inlineStr">
+        <is>
+          <t>#323</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="5" t="inlineStr">
@@ -8713,11 +9428,16 @@
       </c>
       <c r="J140" s="14" t="inlineStr">
         <is>
-          <t>test/m11-e2e</t>
+          <t>test/m11-1</t>
         </is>
       </c>
       <c r="K140" s="14" t="inlineStr"/>
       <c r="L140" s="14" t="inlineStr"/>
+      <c r="M140" s="15" t="inlineStr">
+        <is>
+          <t>#324</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="5" t="inlineStr">
@@ -8765,11 +9485,16 @@
       </c>
       <c r="J141" s="14" t="inlineStr">
         <is>
-          <t>test/m11-e2e</t>
+          <t>test/m11-2</t>
         </is>
       </c>
       <c r="K141" s="14" t="inlineStr"/>
       <c r="L141" s="14" t="inlineStr"/>
+      <c r="M141" s="15" t="inlineStr">
+        <is>
+          <t>#325</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="5" t="inlineStr">
@@ -8817,11 +9542,16 @@
       </c>
       <c r="J142" s="14" t="inlineStr">
         <is>
-          <t>test/m11-e2e</t>
+          <t>test/m11-3</t>
         </is>
       </c>
       <c r="K142" s="14" t="inlineStr"/>
       <c r="L142" s="14" t="inlineStr"/>
+      <c r="M142" s="15" t="inlineStr">
+        <is>
+          <t>#326</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="5" t="inlineStr">
@@ -8869,11 +9599,16 @@
       </c>
       <c r="J143" s="14" t="inlineStr">
         <is>
-          <t>test/m11-e2e</t>
+          <t>test/m11-4</t>
         </is>
       </c>
       <c r="K143" s="14" t="inlineStr"/>
       <c r="L143" s="14" t="inlineStr"/>
+      <c r="M143" s="15" t="inlineStr">
+        <is>
+          <t>#327</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="5" t="inlineStr">
@@ -8921,11 +9656,16 @@
       </c>
       <c r="J144" s="14" t="inlineStr">
         <is>
-          <t>test/m11-e2e</t>
+          <t>test/m11-5</t>
         </is>
       </c>
       <c r="K144" s="14" t="inlineStr"/>
       <c r="L144" s="14" t="inlineStr"/>
+      <c r="M144" s="15" t="inlineStr">
+        <is>
+          <t>#328</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="5" t="inlineStr">
@@ -8973,11 +9713,16 @@
       </c>
       <c r="J145" s="14" t="inlineStr">
         <is>
-          <t>test/m11-e2e</t>
+          <t>test/m11-6</t>
         </is>
       </c>
       <c r="K145" s="14" t="inlineStr"/>
       <c r="L145" s="14" t="inlineStr"/>
+      <c r="M145" s="15" t="inlineStr">
+        <is>
+          <t>#329</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="5" t="inlineStr">
@@ -9025,11 +9770,16 @@
       </c>
       <c r="J146" s="14" t="inlineStr">
         <is>
-          <t>test/m11-e2e</t>
+          <t>test/m11-7</t>
         </is>
       </c>
       <c r="K146" s="14" t="inlineStr"/>
       <c r="L146" s="14" t="inlineStr"/>
+      <c r="M146" s="15" t="inlineStr">
+        <is>
+          <t>#330</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="5" t="inlineStr">
@@ -9077,11 +9827,16 @@
       </c>
       <c r="J147" s="14" t="inlineStr">
         <is>
-          <t>test/m11-e2e</t>
+          <t>test/m11-8</t>
         </is>
       </c>
       <c r="K147" s="14" t="inlineStr"/>
       <c r="L147" s="14" t="inlineStr"/>
+      <c r="M147" s="15" t="inlineStr">
+        <is>
+          <t>#331</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="5" t="inlineStr">
@@ -9129,11 +9884,16 @@
       </c>
       <c r="J148" s="14" t="inlineStr">
         <is>
-          <t>test/m11-e2e</t>
+          <t>test/m11-9</t>
         </is>
       </c>
       <c r="K148" s="14" t="inlineStr"/>
       <c r="L148" s="14" t="inlineStr"/>
+      <c r="M148" s="15" t="inlineStr">
+        <is>
+          <t>#332</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="5" t="inlineStr">
@@ -9181,11 +9941,16 @@
       </c>
       <c r="J149" s="14" t="inlineStr">
         <is>
-          <t>test/m11-e2e</t>
+          <t>test/m11-10</t>
         </is>
       </c>
       <c r="K149" s="14" t="inlineStr"/>
       <c r="L149" s="14" t="inlineStr"/>
+      <c r="M149" s="15" t="inlineStr">
+        <is>
+          <t>#333</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="5" t="inlineStr">
@@ -9233,11 +9998,16 @@
       </c>
       <c r="J150" s="14" t="inlineStr">
         <is>
-          <t>chore/m12-hardening</t>
+          <t>chore/m12-1</t>
         </is>
       </c>
       <c r="K150" s="14" t="inlineStr"/>
       <c r="L150" s="14" t="inlineStr"/>
+      <c r="M150" s="15" t="inlineStr">
+        <is>
+          <t>#334</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="5" t="inlineStr">
@@ -9285,11 +10055,16 @@
       </c>
       <c r="J151" s="14" t="inlineStr">
         <is>
-          <t>chore/m12-hardening</t>
+          <t>chore/m12-2</t>
         </is>
       </c>
       <c r="K151" s="14" t="inlineStr"/>
       <c r="L151" s="14" t="inlineStr"/>
+      <c r="M151" s="15" t="inlineStr">
+        <is>
+          <t>#335</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="5" t="inlineStr">
@@ -9337,11 +10112,16 @@
       </c>
       <c r="J152" s="14" t="inlineStr">
         <is>
-          <t>chore/m12-hardening</t>
+          <t>chore/m12-3</t>
         </is>
       </c>
       <c r="K152" s="14" t="inlineStr"/>
       <c r="L152" s="14" t="inlineStr"/>
+      <c r="M152" s="15" t="inlineStr">
+        <is>
+          <t>#336</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="5" t="inlineStr">
@@ -9389,11 +10169,16 @@
       </c>
       <c r="J153" s="14" t="inlineStr">
         <is>
-          <t>chore/m12-hardening</t>
+          <t>chore/m12-4</t>
         </is>
       </c>
       <c r="K153" s="14" t="inlineStr"/>
       <c r="L153" s="14" t="inlineStr"/>
+      <c r="M153" s="15" t="inlineStr">
+        <is>
+          <t>#337</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="5" t="inlineStr">
@@ -9441,11 +10226,16 @@
       </c>
       <c r="J154" s="14" t="inlineStr">
         <is>
-          <t>chore/m12-hardening</t>
+          <t>chore/m12-5</t>
         </is>
       </c>
       <c r="K154" s="14" t="inlineStr"/>
       <c r="L154" s="14" t="inlineStr"/>
+      <c r="M154" s="15" t="inlineStr">
+        <is>
+          <t>#338</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="5" t="inlineStr">
@@ -9493,11 +10283,16 @@
       </c>
       <c r="J155" s="14" t="inlineStr">
         <is>
-          <t>chore/m12-hardening</t>
+          <t>chore/m12-6</t>
         </is>
       </c>
       <c r="K155" s="14" t="inlineStr"/>
       <c r="L155" s="14" t="inlineStr"/>
+      <c r="M155" s="15" t="inlineStr">
+        <is>
+          <t>#339</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="5" t="inlineStr">
@@ -9545,11 +10340,16 @@
       </c>
       <c r="J156" s="14" t="inlineStr">
         <is>
-          <t>chore/m12-hardening</t>
+          <t>chore/m12-7</t>
         </is>
       </c>
       <c r="K156" s="14" t="inlineStr"/>
       <c r="L156" s="14" t="inlineStr"/>
+      <c r="M156" s="15" t="inlineStr">
+        <is>
+          <t>#340</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="5" t="inlineStr">
@@ -9597,11 +10397,16 @@
       </c>
       <c r="J157" s="14" t="inlineStr">
         <is>
-          <t>chore/m12-hardening</t>
+          <t>chore/m12-8</t>
         </is>
       </c>
       <c r="K157" s="14" t="inlineStr"/>
       <c r="L157" s="14" t="inlineStr"/>
+      <c r="M157" s="15" t="inlineStr">
+        <is>
+          <t>#341</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="5" t="inlineStr">
@@ -9649,11 +10454,16 @@
       </c>
       <c r="J158" s="14" t="inlineStr">
         <is>
-          <t>release/m13-launch</t>
+          <t>release/m13-1</t>
         </is>
       </c>
       <c r="K158" s="14" t="inlineStr"/>
       <c r="L158" s="14" t="inlineStr"/>
+      <c r="M158" s="15" t="inlineStr">
+        <is>
+          <t>#342</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="5" t="inlineStr">
@@ -9701,11 +10511,16 @@
       </c>
       <c r="J159" s="14" t="inlineStr">
         <is>
-          <t>release/m13-launch</t>
+          <t>release/m13-2</t>
         </is>
       </c>
       <c r="K159" s="14" t="inlineStr"/>
       <c r="L159" s="14" t="inlineStr"/>
+      <c r="M159" s="15" t="inlineStr">
+        <is>
+          <t>#343</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="5" t="inlineStr">
@@ -9753,11 +10568,16 @@
       </c>
       <c r="J160" s="14" t="inlineStr">
         <is>
-          <t>release/m13-launch</t>
+          <t>release/m13-3</t>
         </is>
       </c>
       <c r="K160" s="14" t="inlineStr"/>
       <c r="L160" s="14" t="inlineStr"/>
+      <c r="M160" s="15" t="inlineStr">
+        <is>
+          <t>#344</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="5" t="inlineStr">
@@ -9805,11 +10625,16 @@
       </c>
       <c r="J161" s="14" t="inlineStr">
         <is>
-          <t>release/m13-launch</t>
+          <t>release/m13-4</t>
         </is>
       </c>
       <c r="K161" s="14" t="inlineStr"/>
       <c r="L161" s="14" t="inlineStr"/>
+      <c r="M161" s="15" t="inlineStr">
+        <is>
+          <t>#345</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="5" t="inlineStr">
@@ -9857,11 +10682,16 @@
       </c>
       <c r="J162" s="14" t="inlineStr">
         <is>
-          <t>release/m13-launch</t>
+          <t>release/m13-5</t>
         </is>
       </c>
       <c r="K162" s="14" t="inlineStr"/>
       <c r="L162" s="14" t="inlineStr"/>
+      <c r="M162" s="15" t="inlineStr">
+        <is>
+          <t>#346</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="5" t="inlineStr">
@@ -9909,11 +10739,16 @@
       </c>
       <c r="J163" s="14" t="inlineStr">
         <is>
-          <t>release/m13-launch</t>
+          <t>release/m13-8</t>
         </is>
       </c>
       <c r="K163" s="14" t="inlineStr"/>
       <c r="L163" s="14" t="inlineStr"/>
+      <c r="M163" s="15" t="inlineStr">
+        <is>
+          <t>#347</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="5" t="inlineStr">
@@ -9961,11 +10796,16 @@
       </c>
       <c r="J164" s="14" t="inlineStr">
         <is>
-          <t>release/m13-launch</t>
+          <t>release/m13-6</t>
         </is>
       </c>
       <c r="K164" s="14" t="inlineStr"/>
       <c r="L164" s="14" t="inlineStr"/>
+      <c r="M164" s="15" t="inlineStr">
+        <is>
+          <t>#348</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="5" t="inlineStr">
@@ -10013,14 +10853,19 @@
       </c>
       <c r="J165" s="14" t="inlineStr">
         <is>
-          <t>release/m13-launch</t>
+          <t>release/m13-7</t>
         </is>
       </c>
       <c r="K165" s="14" t="inlineStr"/>
       <c r="L165" s="14" t="inlineStr"/>
+      <c r="M165" s="15" t="inlineStr">
+        <is>
+          <t>#349</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L165"/>
+  <autoFilter ref="A1:M165"/>
   <conditionalFormatting sqref="I2:I165">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"✅ مكتمل"</formula>
@@ -10037,6 +10882,172 @@
       <formula1>"⬜ لم يبدأ,🟨 قيد التنفيذ,✅ مكتمل,⛔ متوقف"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M115" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M129" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M130" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M131" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M132" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M133" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M134" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M135" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M136" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M137" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M138" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M139" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M140" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M141" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M142" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M143" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M144" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M145" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M146" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M147" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M148" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M149" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M150" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M151" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M152" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M153" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M154" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M155" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M156" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M157" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M158" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M159" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M160" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M161" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M162" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M163" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M164" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M165" r:id="rId164"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10073,166 +11084,166 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="B2" s="16">
+      <c r="B2" s="17">
         <f>SUMIFS(Tasks!$G$2:$G$165,Tasks!$F$2:$F$165,A2)</f>
         <v/>
       </c>
-      <c r="C2" s="17">
+      <c r="C2" s="18">
         <f>IFERROR(B2/SUM($B$2:$B$12),0)</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>BE+FE</t>
         </is>
       </c>
-      <c r="B3" s="16">
+      <c r="B3" s="17">
         <f>SUMIFS(Tasks!$G$2:$G$165,Tasks!$F$2:$F$165,A3)</f>
         <v/>
       </c>
-      <c r="C3" s="17">
+      <c r="C3" s="18">
         <f>IFERROR(B3/SUM($B$2:$B$12),0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>BE+Ops</t>
         </is>
       </c>
-      <c r="B4" s="16">
+      <c r="B4" s="17">
         <f>SUMIFS(Tasks!$G$2:$G$165,Tasks!$F$2:$F$165,A4)</f>
         <v/>
       </c>
-      <c r="C4" s="17">
+      <c r="C4" s="18">
         <f>IFERROR(B4/SUM($B$2:$B$12),0)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="B5" s="16">
+      <c r="B5" s="17">
         <f>SUMIFS(Tasks!$G$2:$G$165,Tasks!$F$2:$F$165,A5)</f>
         <v/>
       </c>
-      <c r="C5" s="17">
+      <c r="C5" s="18">
         <f>IFERROR(B5/SUM($B$2:$B$12),0)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>FE+PM</t>
         </is>
       </c>
-      <c r="B6" s="16">
+      <c r="B6" s="17">
         <f>SUMIFS(Tasks!$G$2:$G$165,Tasks!$F$2:$F$165,A6)</f>
         <v/>
       </c>
-      <c r="C6" s="17">
+      <c r="C6" s="18">
         <f>IFERROR(B6/SUM($B$2:$B$12),0)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Ops</t>
         </is>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="17">
         <f>SUMIFS(Tasks!$G$2:$G$165,Tasks!$F$2:$F$165,A7)</f>
         <v/>
       </c>
-      <c r="C7" s="17">
+      <c r="C7" s="18">
         <f>IFERROR(B7/SUM($B$2:$B$12),0)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>PM</t>
         </is>
       </c>
-      <c r="B8" s="16">
+      <c r="B8" s="17">
         <f>SUMIFS(Tasks!$G$2:$G$165,Tasks!$F$2:$F$165,A8)</f>
         <v/>
       </c>
-      <c r="C8" s="17">
+      <c r="C8" s="18">
         <f>IFERROR(B8/SUM($B$2:$B$12),0)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>PM+BE</t>
         </is>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="17">
         <f>SUMIFS(Tasks!$G$2:$G$165,Tasks!$F$2:$F$165,A9)</f>
         <v/>
       </c>
-      <c r="C9" s="17">
+      <c r="C9" s="18">
         <f>IFERROR(B9/SUM($B$2:$B$12),0)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>PM+QA</t>
         </is>
       </c>
-      <c r="B10" s="16">
+      <c r="B10" s="17">
         <f>SUMIFS(Tasks!$G$2:$G$165,Tasks!$F$2:$F$165,A10)</f>
         <v/>
       </c>
-      <c r="C10" s="17">
+      <c r="C10" s="18">
         <f>IFERROR(B10/SUM($B$2:$B$12),0)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>QA</t>
         </is>
       </c>
-      <c r="B11" s="16">
+      <c r="B11" s="17">
         <f>SUMIFS(Tasks!$G$2:$G$165,Tasks!$F$2:$F$165,A11)</f>
         <v/>
       </c>
-      <c r="C11" s="17">
+      <c r="C11" s="18">
         <f>IFERROR(B11/SUM($B$2:$B$12),0)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>الكل</t>
         </is>
       </c>
-      <c r="B12" s="16">
+      <c r="B12" s="17">
         <f>SUMIFS(Tasks!$G$2:$G$165,Tasks!$F$2:$F$165,A12)</f>
         <v/>
       </c>
-      <c r="C12" s="17">
+      <c r="C12" s="18">
         <f>IFERROR(B12/SUM($B$2:$B$12),0)</f>
         <v/>
       </c>

</xml_diff>